<commit_message>
Add Phase II, remediation, and reclamation verticals with render optimizations.
Extend profiles, narratives, checklists, samples, and E2E scripts for Phase II ESA, groundwater, Phase III remediation, and reclamation certificates; reduce duplicate Excel/template work on preflight and batch render.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/samples/groundwater_monitoring_data.xlsx
+++ b/samples/groundwater_monitoring_data.xlsx
@@ -12,6 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WaterLevels" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GroundwaterLab" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldNotes" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PhraseCatalog" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -417,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:V2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -491,6 +492,46 @@
           <t>site_map_image_path</t>
         </is>
       </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>gw_program_intro_selected</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>gw_sampling_methods_selected</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>gw_data_usability_selected</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>gw_recommendations_selected</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>gw_program_intro</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>gw_sampling_methods</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>gw_data_usability</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>gw_recommendations</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -547,6 +588,46 @@
       </c>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>low_flow</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>usable</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>investigate</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>This report presents results of the annual groundwater monitoring program conducted to assess groundwater quality and water levels relative to applicable Alberta guidelines and site-specific objectives.</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>Groundwater samples were collected using low-flow purging and sampling methods in accordance with project-specific sampling procedures and laboratory requirements.</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>Field notes and laboratory quality control indicate that the groundwater data are suitable for comparison to applicable guidelines, subject to the limitations noted herein.</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>Ecoventure recommends additional investigation of exceedances identified in this reporting period, including potential source areas and downgradient wells.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -764,7 +845,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -849,7 +930,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2025-04-15</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -859,7 +940,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>380</t>
+          <t>280</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -891,25 +972,62 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t>Chloride</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>380</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>mg/L</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>MW-2</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
           <t>Benzene</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>0.0005</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>mg/L</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>0.005</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -976,4 +1094,375 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>phrase_key</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>option_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>closure_recommendation</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>support_closure</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Based on the data presented, Ecoventure supports proceeding with regulatory closure documentation, subject to agency review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>closure_recommendation</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>defer</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Ecoventure recommends deferring closure until additional monitoring or remedial work is completed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>confirmatory_summary</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>met</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Confirmatory sampling results indicate that remedial objectives were met for the parameters and media evaluated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>confirmatory_summary</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>not_met</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Confirmatory sampling results indicate that additional remedial action or monitoring is required for one or more parameters.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>drilling_waste_intro</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>option_1_aer</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Drilling waste was managed in accordance with AER requirements. Option 1 (AER, 2014) applies to this well.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>drilling_waste_intro</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>option_2</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Drilling waste was managed under an approved alternative disposal pathway. Details are summarized in the drilling waste table.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>gw_data_usability</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>usable</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Field notes and laboratory quality control indicate that the groundwater data are suitable for comparison to applicable guidelines, subject to the limitations noted herein.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>gw_data_usability</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>qualified</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Some data limitations are noted in the field log and tables below; interpreted trends should be considered qualified where purge volumes or hold times were atypical.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>gw_program_intro</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>This report presents results of the annual groundwater monitoring program conducted to assess groundwater quality and water levels relative to applicable Alberta guidelines and site-specific objectives.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>gw_program_intro</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>This report summarizes baseline groundwater quality and static water levels following installation of the monitoring well network.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>gw_recommendations</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>continue</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Ecoventure recommends continued groundwater monitoring at the established frequency to evaluate temporal trends and confirm stability of exceedances.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>gw_recommendations</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>investigate</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Ecoventure recommends additional investigation of exceedances identified in this reporting period, including potential source areas and downgradient wells.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>gw_sampling_methods</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>low_flow</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Groundwater samples were collected using low-flow purging and sampling methods in accordance with project-specific sampling procedures and laboratory requirements.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>gw_sampling_methods</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>bailer</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Groundwater samples were collected after purging each monitoring well until field parameters stabilized, using dedicated sampling equipment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>phase2_recommendation</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>recommended</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Based on the findings of this Phase I ESA, a Phase II Environmental Site Assessment is recommended to further evaluate identified areas of potential environmental concern.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>phase2_recommendation</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>not_required</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Based on the findings of this Phase I ESA, a Phase II Environmental Site Assessment is not recommended at this time, subject to client direction and future land use.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>remediation_status</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ongoing</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Remediation activities are ongoing at the site under an approved remedial action plan. This report summarizes confirmatory sampling and progress toward remedial objectives.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>remediation_status</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>confirmatory</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>This report documents confirmatory groundwater and soil sampling conducted to verify achievement of remedial objectives.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>site_recon_intro</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>not_completed</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>A site visit was not completed as part of this Phase I ESA. Findings are based on available records, regulatory databases, and historical air photo review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>site_recon_intro</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>A site visit was completed as part of this Phase I ESA. Observations from the visit are summarized below and in the site visit checklist.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add DWDA compliance, unified render_service, and docs/rules sync.
Unify Streamlit, CLI, and project-folder rendering through render_service with appendix-aware SED/DWDA enrichment, compliance manifest snapshots, and qp_checklists in deliverable zip. Add Ecoventure workbook ingest, 284-test suite with count guard, Windows CI smoke job, and scoped DWDA Cursor rule.
</commit_message>
<xml_diff>
--- a/samples/groundwater_monitoring_data.xlsx
+++ b/samples/groundwater_monitoring_data.xlsx
@@ -1102,7 +1102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1220,243 +1220,311 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Drilling waste was managed under an approved alternative disposal pathway. Details are summarized in the drilling waste table.</t>
+          <t>Drilling waste was managed under Checklist Compliance Option 2. Calculation tables are provided in Appendix G.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>gw_data_usability</t>
+          <t>drilling_waste_intro</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>usable</t>
+          <t>option_3</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Field notes and laboratory quality control indicate that the groundwater data are suitable for comparison to applicable guidelines, subject to the limitations noted herein.</t>
+          <t>Drilling waste disposal areas were assessed under Compliance Option 3 per Assessing Drilling Waste Disposal Areas guidance.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>gw_data_usability</t>
+          <t>drilling_waste_intro</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>qualified</t>
+          <t>approved_facility</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Some data limitations are noted in the field log and tables below; interpreted trends should be considered qualified where purge volumes or hold times were atypical.</t>
+          <t>All drilling waste was managed at an AER-approved waste management facility. On-lease DWDA assessment is limited to documentation review.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>gw_program_intro</t>
+          <t>dwda_salinity_note</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>annual</t>
+          <t>equivalent_salinity</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>This report presents results of the annual groundwater monitoring program conducted to assess groundwater quality and water levels relative to applicable Alberta guidelines and site-specific objectives.</t>
+          <t>Salinity within each drilling waste disposal area may be assessed using Equivalent Salinity Guidelines. Hydrocarbons, metals, and other contaminants within the DWDA and across the remainder of the lease must meet Alberta Tier 1 or Tier 2 remediation guidelines.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>gw_program_intro</t>
+          <t>dwda_salinity_note</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>baseline</t>
+          <t>pending_phase2</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>This report summarizes baseline groundwater quality and static water levels following installation of the monitoring well network.</t>
+          <t>Salinity and other contaminants within identified disposal areas require Phase II sampling and comparison to Equivalent Salinity (salinity) and Alberta Tier 1/2 guidelines (other parameters) before reclamation certification.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>gw_recommendations</t>
+          <t>gw_data_usability</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>continue</t>
+          <t>usable</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Ecoventure recommends continued groundwater monitoring at the established frequency to evaluate temporal trends and confirm stability of exceedances.</t>
+          <t>Field notes and laboratory quality control indicate that the groundwater data are suitable for comparison to applicable guidelines, subject to the limitations noted herein.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>gw_recommendations</t>
+          <t>gw_data_usability</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>investigate</t>
+          <t>qualified</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Ecoventure recommends additional investigation of exceedances identified in this reporting period, including potential source areas and downgradient wells.</t>
+          <t>Some data limitations are noted in the field log and tables below; interpreted trends should be considered qualified where purge volumes or hold times were atypical.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>gw_sampling_methods</t>
+          <t>gw_program_intro</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>low_flow</t>
+          <t>annual</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Groundwater samples were collected using low-flow purging and sampling methods in accordance with project-specific sampling procedures and laboratory requirements.</t>
+          <t>This report presents results of the annual groundwater monitoring program conducted to assess groundwater quality and water levels relative to applicable Alberta guidelines and site-specific objectives.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>gw_sampling_methods</t>
+          <t>gw_program_intro</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>bailer</t>
+          <t>baseline</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Groundwater samples were collected after purging each monitoring well until field parameters stabilized, using dedicated sampling equipment.</t>
+          <t>This report summarizes baseline groundwater quality and static water levels following installation of the monitoring well network.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>phase2_recommendation</t>
+          <t>gw_recommendations</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>recommended</t>
+          <t>continue</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Based on the findings of this Phase I ESA, a Phase II Environmental Site Assessment is recommended to further evaluate identified areas of potential environmental concern.</t>
+          <t>Ecoventure recommends continued groundwater monitoring at the established frequency to evaluate temporal trends and confirm stability of exceedances.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>phase2_recommendation</t>
+          <t>gw_recommendations</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>not_required</t>
+          <t>investigate</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Based on the findings of this Phase I ESA, a Phase II Environmental Site Assessment is not recommended at this time, subject to client direction and future land use.</t>
+          <t>Ecoventure recommends additional investigation of exceedances identified in this reporting period, including potential source areas and downgradient wells.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>remediation_status</t>
+          <t>gw_sampling_methods</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>ongoing</t>
+          <t>low_flow</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Remediation activities are ongoing at the site under an approved remedial action plan. This report summarizes confirmatory sampling and progress toward remedial objectives.</t>
+          <t>Groundwater samples were collected using low-flow purging and sampling methods in accordance with project-specific sampling procedures and laboratory requirements.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>remediation_status</t>
+          <t>gw_sampling_methods</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>confirmatory</t>
+          <t>bailer</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>This report documents confirmatory groundwater and soil sampling conducted to verify achievement of remedial objectives.</t>
+          <t>Groundwater samples were collected after purging each monitoring well until field parameters stabilized, using dedicated sampling equipment.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>site_recon_intro</t>
+          <t>phase2_recommendation</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>not_completed</t>
+          <t>recommended</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>A site visit was not completed as part of this Phase I ESA. Findings are based on available records, regulatory databases, and historical air photo review.</t>
+          <t>Based on the findings of this Phase I ESA, a Phase II Environmental Site Assessment is recommended to further evaluate identified areas of potential environmental concern.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>phase2_recommendation</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>not_required</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Based on the findings of this Phase I ESA, a Phase II Environmental Site Assessment is not recommended at this time, subject to client direction and future land use.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>remediation_status</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>ongoing</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Remediation activities are ongoing at the site under an approved remedial action plan. This report summarizes confirmatory sampling and progress toward remedial objectives.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>remediation_status</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>confirmatory</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>This report documents confirmatory groundwater and soil sampling conducted to verify achievement of remedial objectives.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t>site_recon_intro</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>not_completed</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>A site visit was not completed as part of this Phase I ESA. Findings are based on available records, regulatory databases, and historical air photo review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>site_recon_intro</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
         <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>A site visit was completed as part of this Phase I ESA. Observations from the visit are summarized below and in the site visit checklist.</t>
         </is>

</xml_diff>